<commit_message>
Atualiza dados de estoque
</commit_message>
<xml_diff>
--- a/data/estoque-022/BD_022.xlsx
+++ b/data/estoque-022/BD_022.xlsx
@@ -1,13 +1,5 @@
 
-<file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <sheets>
-    <sheet name="Plan1" sheetId="1" r:id="rId1"/>
-  </sheets>
-</workbook>
-</file>
-
-<file path=xl/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetData>
     <row r="1" spans="1:54">
@@ -673,12 +665,12 @@
       </c>
       <c r="C5" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[LI00511/26]]></t>
+          <t><![CDATA[LI00513/26]]></t>
         </is>
       </c>
       <c r="D5" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[0400300037]]></t>
+          <t><![CDATA[0400300033]]></t>
         </is>
       </c>
       <c r="E5" t="inlineStr" s="1">
@@ -697,7 +689,7 @@
         </is>
       </c>
       <c r="H5" s="2">
-        <v>1085</v>
+        <v>502</v>
       </c>
       <c r="I5" s="3">
         <v>46270</v>
@@ -772,7 +764,7 @@
       </c>
       <c r="AB5" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[IOG GREGO FRUTAS VERM. 120G - IOGURTE VIÇOSA GREGO FRUTAS VERMELHAS 120G - UNICA - UNICA]]></t>
+          <t><![CDATA[IOG ABACAXI COM COCO 185G - IOGURTE VICOSA ABACAXI COM COCO 185G - UNICA - UNICA]]></t>
         </is>
       </c>
       <c r="AC5" t="inlineStr" s="1">
@@ -807,12 +799,12 @@
       </c>
       <c r="AI5" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[7896706901924]]></t>
+          <t><![CDATA[7896706901672]]></t>
         </is>
       </c>
       <c r="AJ5" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[IOG GREGO FRUTAS VERM. 120G UNICA]]></t>
+          <t><![CDATA[IOG ABACAXI COM COCO 185G UNICA]]></t>
         </is>
       </c>
     </row>
@@ -829,12 +821,12 @@
       </c>
       <c r="C6" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[LI00513/26]]></t>
+          <t><![CDATA[LI00516/26]]></t>
         </is>
       </c>
       <c r="D6" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[0400300033]]></t>
+          <t><![CDATA[0400300015]]></t>
         </is>
       </c>
       <c r="E6" t="inlineStr" s="1">
@@ -853,7 +845,7 @@
         </is>
       </c>
       <c r="H6" s="2">
-        <v>502</v>
+        <v>465</v>
       </c>
       <c r="I6" s="3">
         <v>46270</v>
@@ -928,7 +920,7 @@
       </c>
       <c r="AB6" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[IOG ABACAXI COM COCO 185G - IOGURTE VICOSA ABACAXI COM COCO 185G - UNICA - UNICA]]></t>
+          <t><![CDATA[IOG COCO 185g - IOGURTE VICOSA COCO 185g - UNICA - UNICA]]></t>
         </is>
       </c>
       <c r="AC6" t="inlineStr" s="1">
@@ -963,12 +955,12 @@
       </c>
       <c r="AI6" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[7896706901672]]></t>
+          <t><![CDATA[7896706900637]]></t>
         </is>
       </c>
       <c r="AJ6" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[IOG ABACAXI COM COCO 185G UNICA]]></t>
+          <t><![CDATA[IOG COCO 185g UNICA]]></t>
         </is>
       </c>
     </row>
@@ -1141,12 +1133,12 @@
       </c>
       <c r="C8" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[LI00514/26]]></t>
+          <t><![CDATA[LI00515/26]]></t>
         </is>
       </c>
       <c r="D8" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[0400300041]]></t>
+          <t><![CDATA[0400300023]]></t>
         </is>
       </c>
       <c r="E8" t="inlineStr" s="1">
@@ -1165,7 +1157,7 @@
         </is>
       </c>
       <c r="H8" s="2">
-        <v>1493</v>
+        <v>3581</v>
       </c>
       <c r="I8" s="3">
         <v>46270</v>
@@ -1240,7 +1232,7 @@
       </c>
       <c r="AB8" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[IOG ABACAXI COM COCO 900g - IOGURTE VIÇOSA ABACAXI COM COCO 900g - UNICA - UNICA]]></t>
+          <t><![CDATA[IOG COCO 120g - IOGURTE VICOSA COCO 120g - UNICA - UNICA]]></t>
         </is>
       </c>
       <c r="AC8" t="inlineStr" s="1">
@@ -1275,12 +1267,12 @@
       </c>
       <c r="AI8" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[7896706901894]]></t>
+          <t><![CDATA[7896706904000]]></t>
         </is>
       </c>
       <c r="AJ8" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[IOG ABACAXI COM COCO 900g UNICA]]></t>
+          <t><![CDATA[IOG COCO 120g UNICA]]></t>
         </is>
       </c>
     </row>
@@ -1453,12 +1445,12 @@
       </c>
       <c r="C10" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[LI00516/26]]></t>
+          <t><![CDATA[LI00511/26]]></t>
         </is>
       </c>
       <c r="D10" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[0400300015]]></t>
+          <t><![CDATA[0400300037]]></t>
         </is>
       </c>
       <c r="E10" t="inlineStr" s="1">
@@ -1477,7 +1469,7 @@
         </is>
       </c>
       <c r="H10" s="2">
-        <v>465</v>
+        <v>1085</v>
       </c>
       <c r="I10" s="3">
         <v>46270</v>
@@ -1552,7 +1544,7 @@
       </c>
       <c r="AB10" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[IOG COCO 185g - IOGURTE VICOSA COCO 185g - UNICA - UNICA]]></t>
+          <t><![CDATA[IOG GREGO FRUTAS VERM. 120G - IOGURTE VIÇOSA GREGO FRUTAS VERMELHAS 120G - UNICA - UNICA]]></t>
         </is>
       </c>
       <c r="AC10" t="inlineStr" s="1">
@@ -1587,12 +1579,12 @@
       </c>
       <c r="AI10" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[7896706900637]]></t>
+          <t><![CDATA[7896706901924]]></t>
         </is>
       </c>
       <c r="AJ10" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[IOG COCO 185g UNICA]]></t>
+          <t><![CDATA[IOG GREGO FRUTAS VERM. 120G UNICA]]></t>
         </is>
       </c>
     </row>
@@ -1609,12 +1601,12 @@
       </c>
       <c r="C11" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[LI00515/26]]></t>
+          <t><![CDATA[LI00514/26]]></t>
         </is>
       </c>
       <c r="D11" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[0400300023]]></t>
+          <t><![CDATA[0400300041]]></t>
         </is>
       </c>
       <c r="E11" t="inlineStr" s="1">
@@ -1633,7 +1625,7 @@
         </is>
       </c>
       <c r="H11" s="2">
-        <v>3581</v>
+        <v>1493</v>
       </c>
       <c r="I11" s="3">
         <v>46270</v>
@@ -1708,7 +1700,7 @@
       </c>
       <c r="AB11" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[IOG COCO 120g - IOGURTE VICOSA COCO 120g - UNICA - UNICA]]></t>
+          <t><![CDATA[IOG ABACAXI COM COCO 900g - IOGURTE VIÇOSA ABACAXI COM COCO 900g - UNICA - UNICA]]></t>
         </is>
       </c>
       <c r="AC11" t="inlineStr" s="1">
@@ -1743,12 +1735,12 @@
       </c>
       <c r="AI11" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[7896706904000]]></t>
+          <t><![CDATA[7896706901894]]></t>
         </is>
       </c>
       <c r="AJ11" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[IOG COCO 120g UNICA]]></t>
+          <t><![CDATA[IOG ABACAXI COM COCO 900g UNICA]]></t>
         </is>
       </c>
     </row>
@@ -1765,12 +1757,12 @@
       </c>
       <c r="C12" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[LI00521/26]]></t>
+          <t><![CDATA[LI00519/26]]></t>
         </is>
       </c>
       <c r="D12" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[0400300039]]></t>
+          <t><![CDATA[0400300007]]></t>
         </is>
       </c>
       <c r="E12" t="inlineStr" s="1">
@@ -1789,7 +1781,7 @@
         </is>
       </c>
       <c r="H12" s="2">
-        <v>1630</v>
+        <v>957</v>
       </c>
       <c r="I12" s="3">
         <v>46271</v>
@@ -1864,7 +1856,7 @@
       </c>
       <c r="AB12" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[IOG COCO 900g - IOGURTE VIÇOSA COCO 900g - UNICA - UNICA]]></t>
+          <t><![CDATA[IOG MORANGO 185g - IOGURTE VICOSA MORANGO 185g - UNICA - UNICA]]></t>
         </is>
       </c>
       <c r="AC12" t="inlineStr" s="1">
@@ -1899,12 +1891,12 @@
       </c>
       <c r="AI12" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[7896706901870]]></t>
+          <t><![CDATA[7896706900613]]></t>
         </is>
       </c>
       <c r="AJ12" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[IOG COCO 900g UNICA]]></t>
+          <t><![CDATA[IOG MORANGO 185g UNICA]]></t>
         </is>
       </c>
     </row>
@@ -2077,12 +2069,12 @@
       </c>
       <c r="C14" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[LI00520/26]]></t>
+          <t><![CDATA[LI00521/26]]></t>
         </is>
       </c>
       <c r="D14" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[0400300038]]></t>
+          <t><![CDATA[0400300039]]></t>
         </is>
       </c>
       <c r="E14" t="inlineStr" s="1">
@@ -2101,7 +2093,7 @@
         </is>
       </c>
       <c r="H14" s="2">
-        <v>1088</v>
+        <v>1630</v>
       </c>
       <c r="I14" s="3">
         <v>46271</v>
@@ -2176,7 +2168,7 @@
       </c>
       <c r="AB14" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[IOG MORANGO 900g - IOGURTE VIÇOSA MORANGO 900g - UNICA - UNICA]]></t>
+          <t><![CDATA[IOG COCO 900g - IOGURTE VIÇOSA COCO 900g - UNICA - UNICA]]></t>
         </is>
       </c>
       <c r="AC14" t="inlineStr" s="1">
@@ -2211,12 +2203,12 @@
       </c>
       <c r="AI14" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[7896706901856]]></t>
+          <t><![CDATA[7896706901870]]></t>
         </is>
       </c>
       <c r="AJ14" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[IOG MORANGO 900g UNICA]]></t>
+          <t><![CDATA[IOG COCO 900g UNICA]]></t>
         </is>
       </c>
     </row>
@@ -2233,12 +2225,12 @@
       </c>
       <c r="C15" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[LI00518/26]]></t>
+          <t><![CDATA[LI00520/26]]></t>
         </is>
       </c>
       <c r="D15" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[0400300019]]></t>
+          <t><![CDATA[0400300038]]></t>
         </is>
       </c>
       <c r="E15" t="inlineStr" s="1">
@@ -2257,7 +2249,7 @@
         </is>
       </c>
       <c r="H15" s="2">
-        <v>5888</v>
+        <v>1088</v>
       </c>
       <c r="I15" s="3">
         <v>46271</v>
@@ -2332,7 +2324,7 @@
       </c>
       <c r="AB15" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[IOG MORANGO 120g - IOGURTE VICOSA MORANGO 120g - UNICA - UNICA]]></t>
+          <t><![CDATA[IOG MORANGO 900g - IOGURTE VIÇOSA MORANGO 900g - UNICA - UNICA]]></t>
         </is>
       </c>
       <c r="AC15" t="inlineStr" s="1">
@@ -2367,12 +2359,12 @@
       </c>
       <c r="AI15" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[7896706901009]]></t>
+          <t><![CDATA[7896706901856]]></t>
         </is>
       </c>
       <c r="AJ15" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[IOG MORANGO 120g UNICA]]></t>
+          <t><![CDATA[IOG MORANGO 900g UNICA]]></t>
         </is>
       </c>
     </row>
@@ -2389,12 +2381,12 @@
       </c>
       <c r="C16" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[LI00519/26]]></t>
+          <t><![CDATA[LI00518/26]]></t>
         </is>
       </c>
       <c r="D16" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[0400300007]]></t>
+          <t><![CDATA[0400300019]]></t>
         </is>
       </c>
       <c r="E16" t="inlineStr" s="1">
@@ -2413,7 +2405,7 @@
         </is>
       </c>
       <c r="H16" s="2">
-        <v>957</v>
+        <v>5888</v>
       </c>
       <c r="I16" s="3">
         <v>46271</v>
@@ -2488,7 +2480,7 @@
       </c>
       <c r="AB16" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[IOG MORANGO 185g - IOGURTE VICOSA MORANGO 185g - UNICA - UNICA]]></t>
+          <t><![CDATA[IOG MORANGO 120g - IOGURTE VICOSA MORANGO 120g - UNICA - UNICA]]></t>
         </is>
       </c>
       <c r="AC16" t="inlineStr" s="1">
@@ -2523,12 +2515,12 @@
       </c>
       <c r="AI16" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[7896706900613]]></t>
+          <t><![CDATA[7896706901009]]></t>
         </is>
       </c>
       <c r="AJ16" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[IOG MORANGO 185g UNICA]]></t>
+          <t><![CDATA[IOG MORANGO 120g UNICA]]></t>
         </is>
       </c>
     </row>
@@ -2540,17 +2532,17 @@
       </c>
       <c r="B17" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[005]]></t>
+          <t><![CDATA[009]]></t>
         </is>
       </c>
       <c r="C17" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[LD00265/26]]></t>
+          <t><![CDATA[LR00125/26]]></t>
         </is>
       </c>
       <c r="D17" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[0400500012]]></t>
+          <t><![CDATA[0400900004]]></t>
         </is>
       </c>
       <c r="E17" t="inlineStr" s="1">
@@ -2569,13 +2561,13 @@
         </is>
       </c>
       <c r="H17" s="2">
-        <v>14</v>
+        <v>846</v>
       </c>
       <c r="I17" s="3">
         <v>46314</v>
       </c>
       <c r="J17" s="3">
-        <v>46136</v>
+        <v>46225</v>
       </c>
       <c r="K17" s="2">
         <v>0</v>
@@ -2644,7 +2636,7 @@
       </c>
       <c r="AB17" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[DOCE DE LEITE  C/ CACAU 5KG - DOCE DE LEITE VICOSA C/ CACAU 5KG - FOOD SERVICE - UNICA - UNICA]]></t>
+          <t><![CDATA[CREME DE RICOTA VICOSA 200G - UNICA - UNICA]]></t>
         </is>
       </c>
       <c r="AC17" t="inlineStr" s="1">
@@ -2679,12 +2671,12 @@
       </c>
       <c r="AI17" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[7896706901320]]></t>
+          <t><![CDATA[7896706902020]]></t>
         </is>
       </c>
       <c r="AJ17" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[DOCE DE LEITE  C/ CACAU 5KG UNICA]]></t>
+          <t><![CDATA[CREME DE RICOTA VICOSA 200G UNICA]]></t>
         </is>
       </c>
     </row>
@@ -2696,17 +2688,17 @@
       </c>
       <c r="B18" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[009]]></t>
+          <t><![CDATA[005]]></t>
         </is>
       </c>
       <c r="C18" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[LR00125/26]]></t>
+          <t><![CDATA[LD00265/26]]></t>
         </is>
       </c>
       <c r="D18" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[0400900004]]></t>
+          <t><![CDATA[0400500012]]></t>
         </is>
       </c>
       <c r="E18" t="inlineStr" s="1">
@@ -2725,13 +2717,13 @@
         </is>
       </c>
       <c r="H18" s="2">
-        <v>846</v>
+        <v>14</v>
       </c>
       <c r="I18" s="3">
         <v>46314</v>
       </c>
       <c r="J18" s="3">
-        <v>46225</v>
+        <v>46136</v>
       </c>
       <c r="K18" s="2">
         <v>0</v>
@@ -2800,7 +2792,7 @@
       </c>
       <c r="AB18" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[CREME DE RICOTA VICOSA 200G - UNICA - UNICA]]></t>
+          <t><![CDATA[DOCE DE LEITE  C/ CACAU 5KG - DOCE DE LEITE VICOSA C/ CACAU 5KG - FOOD SERVICE - UNICA - UNICA]]></t>
         </is>
       </c>
       <c r="AC18" t="inlineStr" s="1">
@@ -2835,12 +2827,12 @@
       </c>
       <c r="AI18" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[7896706902020]]></t>
+          <t><![CDATA[7896706901320]]></t>
         </is>
       </c>
       <c r="AJ18" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[CREME DE RICOTA VICOSA 200G UNICA]]></t>
+          <t><![CDATA[DOCE DE LEITE  C/ CACAU 5KG UNICA]]></t>
         </is>
       </c>
     </row>
@@ -3008,17 +3000,17 @@
       </c>
       <c r="B20" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[009]]></t>
+          <t><![CDATA[007]]></t>
         </is>
       </c>
       <c r="C20" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[LR00124/26]]></t>
+          <t><![CDATA[LQ00114/26]]></t>
         </is>
       </c>
       <c r="D20" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[0400900002]]></t>
+          <t><![CDATA[0400700002]]></t>
         </is>
       </c>
       <c r="E20" t="inlineStr" s="1">
@@ -3028,7 +3020,7 @@
       </c>
       <c r="F20" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[UN]]></t>
+          <t><![CDATA[KG]]></t>
         </is>
       </c>
       <c r="G20" t="inlineStr" s="1">
@@ -3037,13 +3029,13 @@
         </is>
       </c>
       <c r="H20" s="2">
-        <v>3515</v>
+        <v>519.541</v>
       </c>
       <c r="I20" s="3">
-        <v>46323</v>
+        <v>46317</v>
       </c>
       <c r="J20" s="3">
-        <v>46224</v>
+        <v>46228</v>
       </c>
       <c r="K20" s="2">
         <v>0</v>
@@ -3112,7 +3104,7 @@
       </c>
       <c r="AB20" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[REQUEIJAO VICOSA 400g - REQUEIJAO VICOSA 400g - UNICA - UNICA]]></t>
+          <t><![CDATA[QUEIJO MUSSARELA VICOSA 3KG COM 2PC - QUEIJO MUSSARELA VICOSA 3KG COM 2PC - UNICA - UNICA]]></t>
         </is>
       </c>
       <c r="AC20" t="inlineStr" s="1">
@@ -3147,12 +3139,12 @@
       </c>
       <c r="AI20" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[7896706900729]]></t>
+          <t><![CDATA[7896706900149]]></t>
         </is>
       </c>
       <c r="AJ20" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[REQUEIJAO VICOSA 400g UNICA]]></t>
+          <t><![CDATA[QUEIJO MUSSARELA VICOSA 3KG COM 2PC UNICA]]></t>
         </is>
       </c>
     </row>
@@ -3320,17 +3312,17 @@
       </c>
       <c r="B22" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[006]]></t>
+          <t><![CDATA[009]]></t>
         </is>
       </c>
       <c r="C22" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[LM00116/26]]></t>
+          <t><![CDATA[LR00124/26]]></t>
         </is>
       </c>
       <c r="D22" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[0400600001]]></t>
+          <t><![CDATA[0400900002]]></t>
         </is>
       </c>
       <c r="E22" t="inlineStr" s="1">
@@ -3349,13 +3341,13 @@
         </is>
       </c>
       <c r="H22" s="2">
-        <v>1200</v>
+        <v>3515</v>
       </c>
       <c r="I22" s="3">
-        <v>46355</v>
+        <v>46323</v>
       </c>
       <c r="J22" s="3">
-        <v>46227</v>
+        <v>46224</v>
       </c>
       <c r="K22" s="2">
         <v>0</v>
@@ -3424,7 +3416,7 @@
       </c>
       <c r="AB22" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[MANTEIGA VICOSA 200g - MANTEIGA VICOSA 200g - UNICA - UNICA]]></t>
+          <t><![CDATA[REQUEIJAO VICOSA 400g - REQUEIJAO VICOSA 400g - UNICA - UNICA]]></t>
         </is>
       </c>
       <c r="AC22" t="inlineStr" s="1">
@@ -3459,12 +3451,12 @@
       </c>
       <c r="AI22" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[7896706900026]]></t>
+          <t><![CDATA[7896706900729]]></t>
         </is>
       </c>
       <c r="AJ22" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[MANTEIGA VICOSA 200g UNICA]]></t>
+          <t><![CDATA[REQUEIJAO VICOSA 400g UNICA]]></t>
         </is>
       </c>
     </row>
@@ -3481,12 +3473,12 @@
       </c>
       <c r="C23" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[LM00117/26]]></t>
+          <t><![CDATA[LM00118/26]]></t>
         </is>
       </c>
       <c r="D23" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[0400600001]]></t>
+          <t><![CDATA[0400600002]]></t>
         </is>
       </c>
       <c r="E23" t="inlineStr" s="1">
@@ -3505,7 +3497,7 @@
         </is>
       </c>
       <c r="H23" s="2">
-        <v>1281</v>
+        <v>504</v>
       </c>
       <c r="I23" s="3">
         <v>46355</v>
@@ -3580,7 +3572,7 @@
       </c>
       <c r="AB23" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[MANTEIGA VICOSA 200g - MANTEIGA VICOSA 200g - UNICA - UNICA]]></t>
+          <t><![CDATA[MANTEIGA VICOSA 500g - MANTEIGA VICOSA 500g - UNICA - UNICA]]></t>
         </is>
       </c>
       <c r="AC23" t="inlineStr" s="1">
@@ -3615,12 +3607,12 @@
       </c>
       <c r="AI23" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[7896706900026]]></t>
+          <t><![CDATA[7896706900712]]></t>
         </is>
       </c>
       <c r="AJ23" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[MANTEIGA VICOSA 200g UNICA]]></t>
+          <t><![CDATA[MANTEIGA VICOSA 500g UNICA]]></t>
         </is>
       </c>
     </row>
@@ -3637,12 +3629,12 @@
       </c>
       <c r="C24" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[LM00118/26]]></t>
+          <t><![CDATA[LM00116/26]]></t>
         </is>
       </c>
       <c r="D24" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[0400600002]]></t>
+          <t><![CDATA[0400600001]]></t>
         </is>
       </c>
       <c r="E24" t="inlineStr" s="1">
@@ -3661,7 +3653,7 @@
         </is>
       </c>
       <c r="H24" s="2">
-        <v>504</v>
+        <v>1200</v>
       </c>
       <c r="I24" s="3">
         <v>46355</v>
@@ -3736,7 +3728,7 @@
       </c>
       <c r="AB24" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[MANTEIGA VICOSA 500g - MANTEIGA VICOSA 500g - UNICA - UNICA]]></t>
+          <t><![CDATA[MANTEIGA VICOSA 200g - MANTEIGA VICOSA 200g - UNICA - UNICA]]></t>
         </is>
       </c>
       <c r="AC24" t="inlineStr" s="1">
@@ -3771,12 +3763,12 @@
       </c>
       <c r="AI24" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[7896706900712]]></t>
+          <t><![CDATA[7896706900026]]></t>
         </is>
       </c>
       <c r="AJ24" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[MANTEIGA VICOSA 500g UNICA]]></t>
+          <t><![CDATA[MANTEIGA VICOSA 200g UNICA]]></t>
         </is>
       </c>
     </row>
@@ -3788,17 +3780,17 @@
       </c>
       <c r="B25" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[005]]></t>
+          <t><![CDATA[006]]></t>
         </is>
       </c>
       <c r="C25" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[LD00417/26]]></t>
+          <t><![CDATA[LM00117/26]]></t>
         </is>
       </c>
       <c r="D25" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[0400500019]]></t>
+          <t><![CDATA[0400600001]]></t>
         </is>
       </c>
       <c r="E25" t="inlineStr" s="1">
@@ -3817,13 +3809,13 @@
         </is>
       </c>
       <c r="H25" s="2">
-        <v>3108</v>
+        <v>1281</v>
       </c>
       <c r="I25" s="3">
-        <v>46364</v>
+        <v>46355</v>
       </c>
       <c r="J25" s="3">
-        <v>46189</v>
+        <v>46227</v>
       </c>
       <c r="K25" s="2">
         <v>0</v>
@@ -3892,7 +3884,7 @@
       </c>
       <c r="AB25" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[DOCE DE LEITE VICOSA ZERO ACUCAR E LACTOSE 400G - UNICA - UNICA]]></t>
+          <t><![CDATA[MANTEIGA VICOSA 200g - MANTEIGA VICOSA 200g - UNICA - UNICA]]></t>
         </is>
       </c>
       <c r="AC25" t="inlineStr" s="1">
@@ -3927,12 +3919,12 @@
       </c>
       <c r="AI25" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[7896706902068]]></t>
+          <t><![CDATA[7896706900026]]></t>
         </is>
       </c>
       <c r="AJ25" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[DOCE DE LEITE VICOSA ZERO ACUCAR E LACTOSE 400G UNICA]]></t>
+          <t><![CDATA[MANTEIGA VICOSA 200g UNICA]]></t>
         </is>
       </c>
     </row>
@@ -3944,17 +3936,17 @@
       </c>
       <c r="B26" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[005]]></t>
+          <t><![CDATA[006]]></t>
         </is>
       </c>
       <c r="C26" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[LD00421/26]]></t>
+          <t><![CDATA[LM00119/26]]></t>
         </is>
       </c>
       <c r="D26" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[0400500008]]></t>
+          <t><![CDATA[0400600001]]></t>
         </is>
       </c>
       <c r="E26" t="inlineStr" s="1">
@@ -3973,13 +3965,13 @@
         </is>
       </c>
       <c r="H26" s="2">
-        <v>3129</v>
+        <v>2143</v>
       </c>
       <c r="I26" s="3">
-        <v>46365</v>
+        <v>46356</v>
       </c>
       <c r="J26" s="3">
-        <v>46188</v>
+        <v>46228</v>
       </c>
       <c r="K26" s="2">
         <v>0</v>
@@ -4048,7 +4040,7 @@
       </c>
       <c r="AB26" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[DOCE DE LEITE VICOSA 800g - DOCE DE LEITE VICOSA 800g - UNICA - UNICA]]></t>
+          <t><![CDATA[MANTEIGA VICOSA 200g - MANTEIGA VICOSA 200g - UNICA - UNICA]]></t>
         </is>
       </c>
       <c r="AC26" t="inlineStr" s="1">
@@ -4083,12 +4075,12 @@
       </c>
       <c r="AI26" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[7896706900019]]></t>
+          <t><![CDATA[7896706900026]]></t>
         </is>
       </c>
       <c r="AJ26" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[DOCE DE LEITE VICOSA 800g UNICA]]></t>
+          <t><![CDATA[MANTEIGA VICOSA 200g UNICA]]></t>
         </is>
       </c>
     </row>
@@ -4100,17 +4092,17 @@
       </c>
       <c r="B27" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[005]]></t>
+          <t><![CDATA[006]]></t>
         </is>
       </c>
       <c r="C27" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[LD00536/26]]></t>
+          <t><![CDATA[LM00121/26]]></t>
         </is>
       </c>
       <c r="D27" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[0400500008]]></t>
+          <t><![CDATA[0400600002]]></t>
         </is>
       </c>
       <c r="E27" t="inlineStr" s="1">
@@ -4129,13 +4121,13 @@
         </is>
       </c>
       <c r="H27" s="2">
-        <v>3151</v>
+        <v>623</v>
       </c>
       <c r="I27" s="3">
-        <v>46403</v>
+        <v>46356</v>
       </c>
       <c r="J27" s="3">
-        <v>46223</v>
+        <v>46228</v>
       </c>
       <c r="K27" s="2">
         <v>0</v>
@@ -4204,7 +4196,7 @@
       </c>
       <c r="AB27" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[DOCE DE LEITE VICOSA 800g - DOCE DE LEITE VICOSA 800g - UNICA - UNICA]]></t>
+          <t><![CDATA[MANTEIGA VICOSA 500g - MANTEIGA VICOSA 500g - UNICA - UNICA]]></t>
         </is>
       </c>
       <c r="AC27" t="inlineStr" s="1">
@@ -4239,12 +4231,12 @@
       </c>
       <c r="AI27" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[7896706900019]]></t>
+          <t><![CDATA[7896706900712]]></t>
         </is>
       </c>
       <c r="AJ27" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[DOCE DE LEITE VICOSA 800g UNICA]]></t>
+          <t><![CDATA[MANTEIGA VICOSA 500g UNICA]]></t>
         </is>
       </c>
     </row>
@@ -4256,17 +4248,17 @@
       </c>
       <c r="B28" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[005]]></t>
+          <t><![CDATA[006]]></t>
         </is>
       </c>
       <c r="C28" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[LD00544/26]]></t>
+          <t><![CDATA[LM00122/26]]></t>
         </is>
       </c>
       <c r="D28" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[0400500004]]></t>
+          <t><![CDATA[0400600002]]></t>
         </is>
       </c>
       <c r="E28" t="inlineStr" s="1">
@@ -4285,13 +4277,13 @@
         </is>
       </c>
       <c r="H28" s="2">
-        <v>6483</v>
+        <v>490</v>
       </c>
       <c r="I28" s="3">
-        <v>46404</v>
+        <v>46357</v>
       </c>
       <c r="J28" s="3">
-        <v>46225</v>
+        <v>46228</v>
       </c>
       <c r="K28" s="2">
         <v>0</v>
@@ -4360,7 +4352,7 @@
       </c>
       <c r="AB28" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[DOCE DE LEITE VICOSA 400g - DOCE DE LEITE VICOSA 400g - UNICA - UNICA]]></t>
+          <t><![CDATA[MANTEIGA VICOSA 500g - MANTEIGA VICOSA 500g - UNICA - UNICA]]></t>
         </is>
       </c>
       <c r="AC28" t="inlineStr" s="1">
@@ -4395,12 +4387,12 @@
       </c>
       <c r="AI28" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[7896706900422]]></t>
+          <t><![CDATA[7896706900712]]></t>
         </is>
       </c>
       <c r="AJ28" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[DOCE DE LEITE VICOSA 400g UNICA]]></t>
+          <t><![CDATA[MANTEIGA VICOSA 500g UNICA]]></t>
         </is>
       </c>
     </row>
@@ -4412,17 +4404,17 @@
       </c>
       <c r="B29" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[005]]></t>
+          <t><![CDATA[006]]></t>
         </is>
       </c>
       <c r="C29" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[LD00543/26]]></t>
+          <t><![CDATA[LM00123/26]]></t>
         </is>
       </c>
       <c r="D29" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[0400500004]]></t>
+          <t><![CDATA[0400600002]]></t>
         </is>
       </c>
       <c r="E29" t="inlineStr" s="1">
@@ -4441,13 +4433,13 @@
         </is>
       </c>
       <c r="H29" s="2">
-        <v>5643</v>
+        <v>540</v>
       </c>
       <c r="I29" s="3">
-        <v>46404</v>
+        <v>46357</v>
       </c>
       <c r="J29" s="3">
-        <v>46225</v>
+        <v>46228</v>
       </c>
       <c r="K29" s="2">
         <v>0</v>
@@ -4516,7 +4508,7 @@
       </c>
       <c r="AB29" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[DOCE DE LEITE VICOSA 400g - DOCE DE LEITE VICOSA 400g - UNICA - UNICA]]></t>
+          <t><![CDATA[MANTEIGA VICOSA 500g - MANTEIGA VICOSA 500g - UNICA - UNICA]]></t>
         </is>
       </c>
       <c r="AC29" t="inlineStr" s="1">
@@ -4551,12 +4543,12 @@
       </c>
       <c r="AI29" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[7896706900422]]></t>
+          <t><![CDATA[7896706900712]]></t>
         </is>
       </c>
       <c r="AJ29" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[DOCE DE LEITE VICOSA 400g UNICA]]></t>
+          <t><![CDATA[MANTEIGA VICOSA 500g UNICA]]></t>
         </is>
       </c>
     </row>
@@ -4568,17 +4560,17 @@
       </c>
       <c r="B30" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[005]]></t>
+          <t><![CDATA[006]]></t>
         </is>
       </c>
       <c r="C30" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[LD00542/26]]></t>
+          <t><![CDATA[LM00124/26]]></t>
         </is>
       </c>
       <c r="D30" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[0400500011]]></t>
+          <t><![CDATA[0400600002]]></t>
         </is>
       </c>
       <c r="E30" t="inlineStr" s="1">
@@ -4597,13 +4589,13 @@
         </is>
       </c>
       <c r="H30" s="2">
-        <v>522</v>
+        <v>480</v>
       </c>
       <c r="I30" s="3">
-        <v>46404</v>
+        <v>46357</v>
       </c>
       <c r="J30" s="3">
-        <v>46225</v>
+        <v>46228</v>
       </c>
       <c r="K30" s="2">
         <v>0</v>
@@ -4672,7 +4664,7 @@
       </c>
       <c r="AB30" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[DOCE DE LEITE VICOSA 5KG - DOCE DE LEITE VICOSA 5KG - FOOD SERVICE - UNICA - UNICA]]></t>
+          <t><![CDATA[MANTEIGA VICOSA 500g - MANTEIGA VICOSA 500g - UNICA - UNICA]]></t>
         </is>
       </c>
       <c r="AC30" t="inlineStr" s="1">
@@ -4707,12 +4699,12 @@
       </c>
       <c r="AI30" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[7896706901306]]></t>
+          <t><![CDATA[7896706900712]]></t>
         </is>
       </c>
       <c r="AJ30" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[DOCE DE LEITE VICOSA 5KG UNICA]]></t>
+          <t><![CDATA[MANTEIGA VICOSA 500g UNICA]]></t>
         </is>
       </c>
     </row>
@@ -4729,7 +4721,7 @@
       </c>
       <c r="C31" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[LD00541/26]]></t>
+          <t><![CDATA[LD00417/26]]></t>
         </is>
       </c>
       <c r="D31" t="inlineStr" s="1">
@@ -4753,13 +4745,13 @@
         </is>
       </c>
       <c r="H31" s="2">
-        <v>5500</v>
+        <v>3108</v>
       </c>
       <c r="I31" s="3">
-        <v>46404</v>
+        <v>46364</v>
       </c>
       <c r="J31" s="3">
-        <v>46224</v>
+        <v>46189</v>
       </c>
       <c r="K31" s="2">
         <v>0</v>
@@ -4885,12 +4877,12 @@
       </c>
       <c r="C32" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[LD00547/26]]></t>
+          <t><![CDATA[LD00421/26]]></t>
         </is>
       </c>
       <c r="D32" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[0400500004]]></t>
+          <t><![CDATA[0400500008]]></t>
         </is>
       </c>
       <c r="E32" t="inlineStr" s="1">
@@ -4909,13 +4901,13 @@
         </is>
       </c>
       <c r="H32" s="2">
-        <v>6643</v>
+        <v>3129</v>
       </c>
       <c r="I32" s="3">
-        <v>46405</v>
+        <v>46365</v>
       </c>
       <c r="J32" s="3">
-        <v>46226</v>
+        <v>46188</v>
       </c>
       <c r="K32" s="2">
         <v>0</v>
@@ -4984,7 +4976,7 @@
       </c>
       <c r="AB32" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[DOCE DE LEITE VICOSA 400g - DOCE DE LEITE VICOSA 400g - UNICA - UNICA]]></t>
+          <t><![CDATA[DOCE DE LEITE VICOSA 800g - DOCE DE LEITE VICOSA 800g - UNICA - UNICA]]></t>
         </is>
       </c>
       <c r="AC32" t="inlineStr" s="1">
@@ -5019,12 +5011,12 @@
       </c>
       <c r="AI32" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[7896706900422]]></t>
+          <t><![CDATA[7896706900019]]></t>
         </is>
       </c>
       <c r="AJ32" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[DOCE DE LEITE VICOSA 400g UNICA]]></t>
+          <t><![CDATA[DOCE DE LEITE VICOSA 800g UNICA]]></t>
         </is>
       </c>
     </row>
@@ -5041,12 +5033,12 @@
       </c>
       <c r="C33" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[LD00548/26]]></t>
+          <t><![CDATA[LD00536/26]]></t>
         </is>
       </c>
       <c r="D33" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[0400500004]]></t>
+          <t><![CDATA[0400500008]]></t>
         </is>
       </c>
       <c r="E33" t="inlineStr" s="1">
@@ -5065,13 +5057,13 @@
         </is>
       </c>
       <c r="H33" s="2">
-        <v>5730</v>
+        <v>3151</v>
       </c>
       <c r="I33" s="3">
-        <v>46405</v>
+        <v>46403</v>
       </c>
       <c r="J33" s="3">
-        <v>46226</v>
+        <v>46223</v>
       </c>
       <c r="K33" s="2">
         <v>0</v>
@@ -5140,7 +5132,7 @@
       </c>
       <c r="AB33" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[DOCE DE LEITE VICOSA 400g - DOCE DE LEITE VICOSA 400g - UNICA - UNICA]]></t>
+          <t><![CDATA[DOCE DE LEITE VICOSA 800g - DOCE DE LEITE VICOSA 800g - UNICA - UNICA]]></t>
         </is>
       </c>
       <c r="AC33" t="inlineStr" s="1">
@@ -5175,12 +5167,12 @@
       </c>
       <c r="AI33" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[7896706900422]]></t>
+          <t><![CDATA[7896706900019]]></t>
         </is>
       </c>
       <c r="AJ33" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[DOCE DE LEITE VICOSA 400g UNICA]]></t>
+          <t><![CDATA[DOCE DE LEITE VICOSA 800g UNICA]]></t>
         </is>
       </c>
     </row>
@@ -5197,7 +5189,7 @@
       </c>
       <c r="C34" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[LD00545/26]]></t>
+          <t><![CDATA[LD00541/26]]></t>
         </is>
       </c>
       <c r="D34" t="inlineStr" s="1">
@@ -5221,13 +5213,13 @@
         </is>
       </c>
       <c r="H34" s="2">
-        <v>5370</v>
+        <v>5500</v>
       </c>
       <c r="I34" s="3">
-        <v>46405</v>
+        <v>46404</v>
       </c>
       <c r="J34" s="3">
-        <v>46225</v>
+        <v>46224</v>
       </c>
       <c r="K34" s="2">
         <v>0</v>
@@ -5353,12 +5345,12 @@
       </c>
       <c r="C35" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[LD00550/26]]></t>
+          <t><![CDATA[LD00542/26]]></t>
         </is>
       </c>
       <c r="D35" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[0400500004]]></t>
+          <t><![CDATA[0400500011]]></t>
         </is>
       </c>
       <c r="E35" t="inlineStr" s="1">
@@ -5377,13 +5369,13 @@
         </is>
       </c>
       <c r="H35" s="2">
-        <v>6168</v>
+        <v>522</v>
       </c>
       <c r="I35" s="3">
-        <v>46406</v>
+        <v>46404</v>
       </c>
       <c r="J35" s="3">
-        <v>46227</v>
+        <v>46225</v>
       </c>
       <c r="K35" s="2">
         <v>0</v>
@@ -5452,7 +5444,7 @@
       </c>
       <c r="AB35" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[DOCE DE LEITE VICOSA 400g - DOCE DE LEITE VICOSA 400g - UNICA - UNICA]]></t>
+          <t><![CDATA[DOCE DE LEITE VICOSA 5KG - DOCE DE LEITE VICOSA 5KG - FOOD SERVICE - UNICA - UNICA]]></t>
         </is>
       </c>
       <c r="AC35" t="inlineStr" s="1">
@@ -5487,12 +5479,12 @@
       </c>
       <c r="AI35" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[7896706900422]]></t>
+          <t><![CDATA[7896706901306]]></t>
         </is>
       </c>
       <c r="AJ35" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[DOCE DE LEITE VICOSA 400g UNICA]]></t>
+          <t><![CDATA[DOCE DE LEITE VICOSA 5KG UNICA]]></t>
         </is>
       </c>
     </row>
@@ -5509,12 +5501,12 @@
       </c>
       <c r="C36" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[LD00551/26]]></t>
+          <t><![CDATA[LD00543/26]]></t>
         </is>
       </c>
       <c r="D36" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[0400500011]]></t>
+          <t><![CDATA[0400500004]]></t>
         </is>
       </c>
       <c r="E36" t="inlineStr" s="1">
@@ -5533,13 +5525,13 @@
         </is>
       </c>
       <c r="H36" s="2">
-        <v>502</v>
+        <v>5643</v>
       </c>
       <c r="I36" s="3">
-        <v>46406</v>
+        <v>46404</v>
       </c>
       <c r="J36" s="3">
-        <v>46227</v>
+        <v>46225</v>
       </c>
       <c r="K36" s="2">
         <v>0</v>
@@ -5608,7 +5600,7 @@
       </c>
       <c r="AB36" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[DOCE DE LEITE VICOSA 5KG - DOCE DE LEITE VICOSA 5KG - FOOD SERVICE - UNICA - UNICA]]></t>
+          <t><![CDATA[DOCE DE LEITE VICOSA 400g - DOCE DE LEITE VICOSA 400g - UNICA - UNICA]]></t>
         </is>
       </c>
       <c r="AC36" t="inlineStr" s="1">
@@ -5643,12 +5635,12 @@
       </c>
       <c r="AI36" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[7896706901306]]></t>
+          <t><![CDATA[7896706900422]]></t>
         </is>
       </c>
       <c r="AJ36" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[DOCE DE LEITE VICOSA 5KG UNICA]]></t>
+          <t><![CDATA[DOCE DE LEITE VICOSA 400g UNICA]]></t>
         </is>
       </c>
     </row>
@@ -5665,12 +5657,12 @@
       </c>
       <c r="C37" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[LD00552/26]]></t>
+          <t><![CDATA[LD00544/26]]></t>
         </is>
       </c>
       <c r="D37" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[0400500019]]></t>
+          <t><![CDATA[0400500004]]></t>
         </is>
       </c>
       <c r="E37" t="inlineStr" s="1">
@@ -5689,13 +5681,13 @@
         </is>
       </c>
       <c r="H37" s="2">
-        <v>4905</v>
+        <v>6483</v>
       </c>
       <c r="I37" s="3">
-        <v>46406</v>
+        <v>46404</v>
       </c>
       <c r="J37" s="3">
-        <v>46227</v>
+        <v>46225</v>
       </c>
       <c r="K37" s="2">
         <v>0</v>
@@ -5764,7 +5756,7 @@
       </c>
       <c r="AB37" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[DOCE DE LEITE VICOSA ZERO ACUCAR E LACTOSE 400G - UNICA - UNICA]]></t>
+          <t><![CDATA[DOCE DE LEITE VICOSA 400g - DOCE DE LEITE VICOSA 400g - UNICA - UNICA]]></t>
         </is>
       </c>
       <c r="AC37" t="inlineStr" s="1">
@@ -5799,12 +5791,12 @@
       </c>
       <c r="AI37" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[7896706902068]]></t>
+          <t><![CDATA[7896706900422]]></t>
         </is>
       </c>
       <c r="AJ37" t="inlineStr" s="1">
         <is>
-          <t><![CDATA[DOCE DE LEITE VICOSA ZERO ACUCAR E LACTOSE 400G UNICA]]></t>
+          <t><![CDATA[DOCE DE LEITE VICOSA 400g UNICA]]></t>
         </is>
       </c>
     </row>
@@ -5821,144 +5813,1704 @@
       </c>
       <c r="C38" t="inlineStr" s="1">
         <is>
+          <t><![CDATA[LD00545/26]]></t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[0400500019]]></t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[U]]></t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[UN]]></t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[022]]></t>
+        </is>
+      </c>
+      <c r="H38" s="2">
+        <v>5370</v>
+      </c>
+      <c r="I38" s="3">
+        <v>46405</v>
+      </c>
+      <c r="J38" s="3">
+        <v>46225</v>
+      </c>
+      <c r="K38" s="2">
+        <v>0</v>
+      </c>
+      <c r="L38" s="2">
+        <v>0</v>
+      </c>
+      <c r="M38" s="2">
+        <v>0</v>
+      </c>
+      <c r="N38" s="2">
+        <v>0</v>
+      </c>
+      <c r="O38" s="2">
+        <v>0</v>
+      </c>
+      <c r="P38" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q38" s="2">
+        <v>0</v>
+      </c>
+      <c r="R38" s="2">
+        <v>0</v>
+      </c>
+      <c r="S38" s="2">
+        <v>0</v>
+      </c>
+      <c r="T38" s="2">
+        <v>0</v>
+      </c>
+      <c r="U38" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="V38" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[2]]></t>
+        </is>
+      </c>
+      <c r="W38" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="X38" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="Y38" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[QUALIDADE]]></t>
+        </is>
+      </c>
+      <c r="Z38" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="AA38" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="AB38" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[DOCE DE LEITE VICOSA ZERO ACUCAR E LACTOSE 400G - UNICA - UNICA]]></t>
+        </is>
+      </c>
+      <c r="AC38" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="AD38" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="AE38" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="AF38" t="inlineStr" s="0">
+        <is>
+          <t><![CDATA[00/00/0000]]></t>
+        </is>
+      </c>
+      <c r="AG38" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="AH38" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="AI38" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[7896706902068]]></t>
+        </is>
+      </c>
+      <c r="AJ38" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[DOCE DE LEITE VICOSA ZERO ACUCAR E LACTOSE 400G UNICA]]></t>
+        </is>
+      </c>
+    </row>
+    <row r="39" spans="1:36">
+      <c r="A39" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[04]]></t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[005]]></t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[LD00547/26]]></t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[0400500004]]></t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[U]]></t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[UN]]></t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[022]]></t>
+        </is>
+      </c>
+      <c r="H39" s="2">
+        <v>6643</v>
+      </c>
+      <c r="I39" s="3">
+        <v>46405</v>
+      </c>
+      <c r="J39" s="3">
+        <v>46226</v>
+      </c>
+      <c r="K39" s="2">
+        <v>0</v>
+      </c>
+      <c r="L39" s="2">
+        <v>0</v>
+      </c>
+      <c r="M39" s="2">
+        <v>0</v>
+      </c>
+      <c r="N39" s="2">
+        <v>0</v>
+      </c>
+      <c r="O39" s="2">
+        <v>0</v>
+      </c>
+      <c r="P39" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q39" s="2">
+        <v>0</v>
+      </c>
+      <c r="R39" s="2">
+        <v>0</v>
+      </c>
+      <c r="S39" s="2">
+        <v>0</v>
+      </c>
+      <c r="T39" s="2">
+        <v>0</v>
+      </c>
+      <c r="U39" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="V39" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[2]]></t>
+        </is>
+      </c>
+      <c r="W39" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="X39" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="Y39" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[QUALIDADE]]></t>
+        </is>
+      </c>
+      <c r="Z39" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="AA39" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="AB39" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[DOCE DE LEITE VICOSA 400g - DOCE DE LEITE VICOSA 400g - UNICA - UNICA]]></t>
+        </is>
+      </c>
+      <c r="AC39" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="AD39" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="AE39" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="AF39" t="inlineStr" s="0">
+        <is>
+          <t><![CDATA[00/00/0000]]></t>
+        </is>
+      </c>
+      <c r="AG39" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="AH39" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="AI39" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[7896706900422]]></t>
+        </is>
+      </c>
+      <c r="AJ39" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[DOCE DE LEITE VICOSA 400g UNICA]]></t>
+        </is>
+      </c>
+    </row>
+    <row r="40" spans="1:36">
+      <c r="A40" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[04]]></t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[005]]></t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[LD00548/26]]></t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[0400500004]]></t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[U]]></t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[UN]]></t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[022]]></t>
+        </is>
+      </c>
+      <c r="H40" s="2">
+        <v>5730</v>
+      </c>
+      <c r="I40" s="3">
+        <v>46405</v>
+      </c>
+      <c r="J40" s="3">
+        <v>46226</v>
+      </c>
+      <c r="K40" s="2">
+        <v>0</v>
+      </c>
+      <c r="L40" s="2">
+        <v>0</v>
+      </c>
+      <c r="M40" s="2">
+        <v>0</v>
+      </c>
+      <c r="N40" s="2">
+        <v>0</v>
+      </c>
+      <c r="O40" s="2">
+        <v>0</v>
+      </c>
+      <c r="P40" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q40" s="2">
+        <v>0</v>
+      </c>
+      <c r="R40" s="2">
+        <v>0</v>
+      </c>
+      <c r="S40" s="2">
+        <v>0</v>
+      </c>
+      <c r="T40" s="2">
+        <v>0</v>
+      </c>
+      <c r="U40" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="V40" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[2]]></t>
+        </is>
+      </c>
+      <c r="W40" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="X40" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="Y40" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[QUALIDADE]]></t>
+        </is>
+      </c>
+      <c r="Z40" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="AA40" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="AB40" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[DOCE DE LEITE VICOSA 400g - DOCE DE LEITE VICOSA 400g - UNICA - UNICA]]></t>
+        </is>
+      </c>
+      <c r="AC40" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="AD40" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="AE40" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="AF40" t="inlineStr" s="0">
+        <is>
+          <t><![CDATA[00/00/0000]]></t>
+        </is>
+      </c>
+      <c r="AG40" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="AH40" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="AI40" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[7896706900422]]></t>
+        </is>
+      </c>
+      <c r="AJ40" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[DOCE DE LEITE VICOSA 400g UNICA]]></t>
+        </is>
+      </c>
+    </row>
+    <row r="41" spans="1:36">
+      <c r="A41" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[04]]></t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[005]]></t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[LD00552/26]]></t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[0400500019]]></t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[U]]></t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[UN]]></t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[022]]></t>
+        </is>
+      </c>
+      <c r="H41" s="2">
+        <v>4905</v>
+      </c>
+      <c r="I41" s="3">
+        <v>46406</v>
+      </c>
+      <c r="J41" s="3">
+        <v>46227</v>
+      </c>
+      <c r="K41" s="2">
+        <v>0</v>
+      </c>
+      <c r="L41" s="2">
+        <v>0</v>
+      </c>
+      <c r="M41" s="2">
+        <v>0</v>
+      </c>
+      <c r="N41" s="2">
+        <v>0</v>
+      </c>
+      <c r="O41" s="2">
+        <v>0</v>
+      </c>
+      <c r="P41" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q41" s="2">
+        <v>0</v>
+      </c>
+      <c r="R41" s="2">
+        <v>0</v>
+      </c>
+      <c r="S41" s="2">
+        <v>0</v>
+      </c>
+      <c r="T41" s="2">
+        <v>0</v>
+      </c>
+      <c r="U41" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="V41" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[2]]></t>
+        </is>
+      </c>
+      <c r="W41" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="X41" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="Y41" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[QUALIDADE]]></t>
+        </is>
+      </c>
+      <c r="Z41" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="AA41" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="AB41" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[DOCE DE LEITE VICOSA ZERO ACUCAR E LACTOSE 400G - UNICA - UNICA]]></t>
+        </is>
+      </c>
+      <c r="AC41" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="AD41" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="AE41" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="AF41" t="inlineStr" s="0">
+        <is>
+          <t><![CDATA[00/00/0000]]></t>
+        </is>
+      </c>
+      <c r="AG41" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="AH41" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="AI41" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[7896706902068]]></t>
+        </is>
+      </c>
+      <c r="AJ41" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[DOCE DE LEITE VICOSA ZERO ACUCAR E LACTOSE 400G UNICA]]></t>
+        </is>
+      </c>
+    </row>
+    <row r="42" spans="1:36">
+      <c r="A42" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[04]]></t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[005]]></t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[LD00551/26]]></t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[0400500011]]></t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[U]]></t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[UN]]></t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[022]]></t>
+        </is>
+      </c>
+      <c r="H42" s="2">
+        <v>502</v>
+      </c>
+      <c r="I42" s="3">
+        <v>46406</v>
+      </c>
+      <c r="J42" s="3">
+        <v>46227</v>
+      </c>
+      <c r="K42" s="2">
+        <v>0</v>
+      </c>
+      <c r="L42" s="2">
+        <v>0</v>
+      </c>
+      <c r="M42" s="2">
+        <v>0</v>
+      </c>
+      <c r="N42" s="2">
+        <v>0</v>
+      </c>
+      <c r="O42" s="2">
+        <v>0</v>
+      </c>
+      <c r="P42" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q42" s="2">
+        <v>0</v>
+      </c>
+      <c r="R42" s="2">
+        <v>0</v>
+      </c>
+      <c r="S42" s="2">
+        <v>0</v>
+      </c>
+      <c r="T42" s="2">
+        <v>0</v>
+      </c>
+      <c r="U42" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="V42" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[2]]></t>
+        </is>
+      </c>
+      <c r="W42" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="X42" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="Y42" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[QUALIDADE]]></t>
+        </is>
+      </c>
+      <c r="Z42" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="AA42" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="AB42" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[DOCE DE LEITE VICOSA 5KG - DOCE DE LEITE VICOSA 5KG - FOOD SERVICE - UNICA - UNICA]]></t>
+        </is>
+      </c>
+      <c r="AC42" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="AD42" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="AE42" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="AF42" t="inlineStr" s="0">
+        <is>
+          <t><![CDATA[00/00/0000]]></t>
+        </is>
+      </c>
+      <c r="AG42" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="AH42" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="AI42" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[7896706901306]]></t>
+        </is>
+      </c>
+      <c r="AJ42" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[DOCE DE LEITE VICOSA 5KG UNICA]]></t>
+        </is>
+      </c>
+    </row>
+    <row r="43" spans="1:36">
+      <c r="A43" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[04]]></t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[005]]></t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[LD00550/26]]></t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[0400500004]]></t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[U]]></t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[UN]]></t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[022]]></t>
+        </is>
+      </c>
+      <c r="H43" s="2">
+        <v>6168</v>
+      </c>
+      <c r="I43" s="3">
+        <v>46406</v>
+      </c>
+      <c r="J43" s="3">
+        <v>46227</v>
+      </c>
+      <c r="K43" s="2">
+        <v>0</v>
+      </c>
+      <c r="L43" s="2">
+        <v>0</v>
+      </c>
+      <c r="M43" s="2">
+        <v>0</v>
+      </c>
+      <c r="N43" s="2">
+        <v>0</v>
+      </c>
+      <c r="O43" s="2">
+        <v>0</v>
+      </c>
+      <c r="P43" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q43" s="2">
+        <v>0</v>
+      </c>
+      <c r="R43" s="2">
+        <v>0</v>
+      </c>
+      <c r="S43" s="2">
+        <v>0</v>
+      </c>
+      <c r="T43" s="2">
+        <v>0</v>
+      </c>
+      <c r="U43" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="V43" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[2]]></t>
+        </is>
+      </c>
+      <c r="W43" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="X43" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="Y43" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[QUALIDADE]]></t>
+        </is>
+      </c>
+      <c r="Z43" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="AA43" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="AB43" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[DOCE DE LEITE VICOSA 400g - DOCE DE LEITE VICOSA 400g - UNICA - UNICA]]></t>
+        </is>
+      </c>
+      <c r="AC43" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="AD43" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="AE43" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="AF43" t="inlineStr" s="0">
+        <is>
+          <t><![CDATA[00/00/0000]]></t>
+        </is>
+      </c>
+      <c r="AG43" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="AH43" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="AI43" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[7896706900422]]></t>
+        </is>
+      </c>
+      <c r="AJ43" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[DOCE DE LEITE VICOSA 400g UNICA]]></t>
+        </is>
+      </c>
+    </row>
+    <row r="44" spans="1:36">
+      <c r="A44" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[04]]></t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[005]]></t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[LD00556/26]]></t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[0400500011]]></t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[U]]></t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[UN]]></t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[022]]></t>
+        </is>
+      </c>
+      <c r="H44" s="2">
+        <v>447</v>
+      </c>
+      <c r="I44" s="3">
+        <v>46407</v>
+      </c>
+      <c r="J44" s="3">
+        <v>46228</v>
+      </c>
+      <c r="K44" s="2">
+        <v>0</v>
+      </c>
+      <c r="L44" s="2">
+        <v>0</v>
+      </c>
+      <c r="M44" s="2">
+        <v>0</v>
+      </c>
+      <c r="N44" s="2">
+        <v>0</v>
+      </c>
+      <c r="O44" s="2">
+        <v>0</v>
+      </c>
+      <c r="P44" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q44" s="2">
+        <v>0</v>
+      </c>
+      <c r="R44" s="2">
+        <v>0</v>
+      </c>
+      <c r="S44" s="2">
+        <v>0</v>
+      </c>
+      <c r="T44" s="2">
+        <v>0</v>
+      </c>
+      <c r="U44" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="V44" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[2]]></t>
+        </is>
+      </c>
+      <c r="W44" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="X44" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="Y44" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[QUALIDADE]]></t>
+        </is>
+      </c>
+      <c r="Z44" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="AA44" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="AB44" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[DOCE DE LEITE VICOSA 5KG - DOCE DE LEITE VICOSA 5KG - FOOD SERVICE - UNICA - UNICA]]></t>
+        </is>
+      </c>
+      <c r="AC44" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="AD44" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="AE44" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="AF44" t="inlineStr" s="0">
+        <is>
+          <t><![CDATA[00/00/0000]]></t>
+        </is>
+      </c>
+      <c r="AG44" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="AH44" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="AI44" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[7896706901306]]></t>
+        </is>
+      </c>
+      <c r="AJ44" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[DOCE DE LEITE VICOSA 5KG UNICA]]></t>
+        </is>
+      </c>
+    </row>
+    <row r="45" spans="1:36">
+      <c r="A45" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[04]]></t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[005]]></t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[LD00557/26]]></t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[0400500011]]></t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[U]]></t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[UN]]></t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[022]]></t>
+        </is>
+      </c>
+      <c r="H45" s="2">
+        <v>512</v>
+      </c>
+      <c r="I45" s="3">
+        <v>46407</v>
+      </c>
+      <c r="J45" s="3">
+        <v>46228</v>
+      </c>
+      <c r="K45" s="2">
+        <v>0</v>
+      </c>
+      <c r="L45" s="2">
+        <v>0</v>
+      </c>
+      <c r="M45" s="2">
+        <v>0</v>
+      </c>
+      <c r="N45" s="2">
+        <v>0</v>
+      </c>
+      <c r="O45" s="2">
+        <v>0</v>
+      </c>
+      <c r="P45" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q45" s="2">
+        <v>0</v>
+      </c>
+      <c r="R45" s="2">
+        <v>0</v>
+      </c>
+      <c r="S45" s="2">
+        <v>0</v>
+      </c>
+      <c r="T45" s="2">
+        <v>0</v>
+      </c>
+      <c r="U45" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="V45" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[2]]></t>
+        </is>
+      </c>
+      <c r="W45" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="X45" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="Y45" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[QUALIDADE]]></t>
+        </is>
+      </c>
+      <c r="Z45" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="AA45" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="AB45" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[DOCE DE LEITE VICOSA 5KG - DOCE DE LEITE VICOSA 5KG - FOOD SERVICE - UNICA - UNICA]]></t>
+        </is>
+      </c>
+      <c r="AC45" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="AD45" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="AE45" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="AF45" t="inlineStr" s="0">
+        <is>
+          <t><![CDATA[00/00/0000]]></t>
+        </is>
+      </c>
+      <c r="AG45" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="AH45" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="AI45" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[7896706901306]]></t>
+        </is>
+      </c>
+      <c r="AJ45" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[DOCE DE LEITE VICOSA 5KG UNICA]]></t>
+        </is>
+      </c>
+    </row>
+    <row r="46" spans="1:36">
+      <c r="A46" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[04]]></t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[005]]></t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[LD00554/26]]></t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[0400500008]]></t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[U]]></t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[UN]]></t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[022]]></t>
+        </is>
+      </c>
+      <c r="H46" s="2">
+        <v>3095</v>
+      </c>
+      <c r="I46" s="3">
+        <v>46407</v>
+      </c>
+      <c r="J46" s="3">
+        <v>46228</v>
+      </c>
+      <c r="K46" s="2">
+        <v>0</v>
+      </c>
+      <c r="L46" s="2">
+        <v>0</v>
+      </c>
+      <c r="M46" s="2">
+        <v>0</v>
+      </c>
+      <c r="N46" s="2">
+        <v>0</v>
+      </c>
+      <c r="O46" s="2">
+        <v>0</v>
+      </c>
+      <c r="P46" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q46" s="2">
+        <v>0</v>
+      </c>
+      <c r="R46" s="2">
+        <v>0</v>
+      </c>
+      <c r="S46" s="2">
+        <v>0</v>
+      </c>
+      <c r="T46" s="2">
+        <v>0</v>
+      </c>
+      <c r="U46" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="V46" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[2]]></t>
+        </is>
+      </c>
+      <c r="W46" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="X46" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="Y46" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[QUALIDADE]]></t>
+        </is>
+      </c>
+      <c r="Z46" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="AA46" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="AB46" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[DOCE DE LEITE VICOSA 800g - DOCE DE LEITE VICOSA 800g - UNICA - UNICA]]></t>
+        </is>
+      </c>
+      <c r="AC46" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="AD46" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="AE46" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="AF46" t="inlineStr" s="0">
+        <is>
+          <t><![CDATA[00/00/0000]]></t>
+        </is>
+      </c>
+      <c r="AG46" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="AH46" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="AI46" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[7896706900019]]></t>
+        </is>
+      </c>
+      <c r="AJ46" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[DOCE DE LEITE VICOSA 800g UNICA]]></t>
+        </is>
+      </c>
+    </row>
+    <row r="47" spans="1:36">
+      <c r="A47" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[04]]></t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[005]]></t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[LD00555/26]]></t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[0400500008]]></t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[U]]></t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[UN]]></t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[022]]></t>
+        </is>
+      </c>
+      <c r="H47" s="2">
+        <v>3372</v>
+      </c>
+      <c r="I47" s="3">
+        <v>46407</v>
+      </c>
+      <c r="J47" s="3">
+        <v>46228</v>
+      </c>
+      <c r="K47" s="2">
+        <v>0</v>
+      </c>
+      <c r="L47" s="2">
+        <v>0</v>
+      </c>
+      <c r="M47" s="2">
+        <v>0</v>
+      </c>
+      <c r="N47" s="2">
+        <v>0</v>
+      </c>
+      <c r="O47" s="2">
+        <v>0</v>
+      </c>
+      <c r="P47" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q47" s="2">
+        <v>0</v>
+      </c>
+      <c r="R47" s="2">
+        <v>0</v>
+      </c>
+      <c r="S47" s="2">
+        <v>0</v>
+      </c>
+      <c r="T47" s="2">
+        <v>0</v>
+      </c>
+      <c r="U47" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="V47" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[2]]></t>
+        </is>
+      </c>
+      <c r="W47" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="X47" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="Y47" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[QUALIDADE]]></t>
+        </is>
+      </c>
+      <c r="Z47" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="AA47" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="AB47" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[DOCE DE LEITE VICOSA 800g - DOCE DE LEITE VICOSA 800g - UNICA - UNICA]]></t>
+        </is>
+      </c>
+      <c r="AC47" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="AD47" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="AE47" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="AF47" t="inlineStr" s="0">
+        <is>
+          <t><![CDATA[00/00/0000]]></t>
+        </is>
+      </c>
+      <c r="AG47" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="AH47" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="AI47" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[7896706900019]]></t>
+        </is>
+      </c>
+      <c r="AJ47" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[DOCE DE LEITE VICOSA 800g UNICA]]></t>
+        </is>
+      </c>
+    </row>
+    <row r="48" spans="1:36">
+      <c r="A48" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[04]]></t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[005]]></t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr" s="1">
+        <is>
           <t><![CDATA[LD00553/26]]></t>
         </is>
       </c>
-      <c r="D38" t="inlineStr" s="1">
+      <c r="D48" t="inlineStr" s="1">
         <is>
           <t><![CDATA[0400500019]]></t>
         </is>
       </c>
-      <c r="E38" t="inlineStr" s="1">
+      <c r="E48" t="inlineStr" s="1">
         <is>
           <t><![CDATA[U]]></t>
         </is>
       </c>
-      <c r="F38" t="inlineStr" s="1">
+      <c r="F48" t="inlineStr" s="1">
         <is>
           <t><![CDATA[UN]]></t>
         </is>
       </c>
-      <c r="G38" t="inlineStr" s="1">
+      <c r="G48" t="inlineStr" s="1">
         <is>
           <t><![CDATA[022]]></t>
         </is>
       </c>
-      <c r="H38" s="2">
+      <c r="H48" s="2">
         <v>5801</v>
       </c>
-      <c r="I38" s="3">
+      <c r="I48" s="3">
         <v>46407</v>
       </c>
-      <c r="J38" s="3">
+      <c r="J48" s="3">
         <v>46227</v>
       </c>
-      <c r="K38" s="2">
-        <v>0</v>
-      </c>
-      <c r="L38" s="2">
-        <v>0</v>
-      </c>
-      <c r="M38" s="2">
-        <v>0</v>
-      </c>
-      <c r="N38" s="2">
-        <v>0</v>
-      </c>
-      <c r="O38" s="2">
-        <v>0</v>
-      </c>
-      <c r="P38" s="2">
-        <v>0</v>
-      </c>
-      <c r="Q38" s="2">
-        <v>0</v>
-      </c>
-      <c r="R38" s="2">
-        <v>0</v>
-      </c>
-      <c r="S38" s="2">
-        <v>0</v>
-      </c>
-      <c r="T38" s="2">
-        <v>0</v>
-      </c>
-      <c r="U38" t="inlineStr" s="1">
-        <is>
-          <t><![CDATA[ ]]></t>
-        </is>
-      </c>
-      <c r="V38" t="inlineStr" s="1">
+      <c r="K48" s="2">
+        <v>0</v>
+      </c>
+      <c r="L48" s="2">
+        <v>0</v>
+      </c>
+      <c r="M48" s="2">
+        <v>0</v>
+      </c>
+      <c r="N48" s="2">
+        <v>0</v>
+      </c>
+      <c r="O48" s="2">
+        <v>0</v>
+      </c>
+      <c r="P48" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q48" s="2">
+        <v>0</v>
+      </c>
+      <c r="R48" s="2">
+        <v>0</v>
+      </c>
+      <c r="S48" s="2">
+        <v>0</v>
+      </c>
+      <c r="T48" s="2">
+        <v>0</v>
+      </c>
+      <c r="U48" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="V48" t="inlineStr" s="1">
         <is>
           <t><![CDATA[2]]></t>
         </is>
       </c>
-      <c r="W38" t="inlineStr" s="1">
-        <is>
-          <t><![CDATA[ ]]></t>
-        </is>
-      </c>
-      <c r="X38" t="inlineStr" s="1">
-        <is>
-          <t><![CDATA[ ]]></t>
-        </is>
-      </c>
-      <c r="Y38" t="inlineStr" s="1">
+      <c r="W48" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="X48" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="Y48" t="inlineStr" s="1">
         <is>
           <t><![CDATA[QUALIDADE]]></t>
         </is>
       </c>
-      <c r="Z38" t="inlineStr" s="1">
-        <is>
-          <t><![CDATA[ ]]></t>
-        </is>
-      </c>
-      <c r="AA38" t="inlineStr" s="1">
-        <is>
-          <t><![CDATA[ ]]></t>
-        </is>
-      </c>
-      <c r="AB38" t="inlineStr" s="1">
+      <c r="Z48" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="AA48" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="AB48" t="inlineStr" s="1">
         <is>
           <t><![CDATA[DOCE DE LEITE VICOSA ZERO ACUCAR E LACTOSE 400G - UNICA - UNICA]]></t>
         </is>
       </c>
-      <c r="AC38" t="inlineStr" s="1">
-        <is>
-          <t><![CDATA[ ]]></t>
-        </is>
-      </c>
-      <c r="AD38" t="inlineStr" s="1">
-        <is>
-          <t><![CDATA[ ]]></t>
-        </is>
-      </c>
-      <c r="AE38" t="inlineStr" s="1">
-        <is>
-          <t><![CDATA[ ]]></t>
-        </is>
-      </c>
-      <c r="AF38" t="inlineStr" s="0">
+      <c r="AC48" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="AD48" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="AE48" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="AF48" t="inlineStr" s="0">
         <is>
           <t><![CDATA[00/00/0000]]></t>
         </is>
       </c>
-      <c r="AG38" t="inlineStr" s="1">
-        <is>
-          <t><![CDATA[ ]]></t>
-        </is>
-      </c>
-      <c r="AH38" t="inlineStr" s="1">
-        <is>
-          <t><![CDATA[ ]]></t>
-        </is>
-      </c>
-      <c r="AI38" t="inlineStr" s="1">
+      <c r="AG48" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="AH48" t="inlineStr" s="1">
+        <is>
+          <t><![CDATA[ ]]></t>
+        </is>
+      </c>
+      <c r="AI48" t="inlineStr" s="1">
         <is>
           <t><![CDATA[7896706902068]]></t>
         </is>
       </c>
-      <c r="AJ38" t="inlineStr" s="1">
+      <c r="AJ48" t="inlineStr" s="1">
         <is>
           <t><![CDATA[DOCE DE LEITE VICOSA ZERO ACUCAR E LACTOSE 400G UNICA]]></t>
         </is>
@@ -5968,7 +7520,7 @@
 </worksheet>
 </file>
 
-<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="2">
     <numFmt numFmtId="166" formatCode="###,###,##0.00000"/>
@@ -6027,4 +7579,12 @@
     <cellStyle name="normal" xfId="0" builtInId="0"/>
   </cellStyles>
 </styleSheet>
+</file>
+
+<file path=xl\workbook.xml><?xml version="1.0" encoding="utf-8"?>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheets>
+    <sheet name="Plan1" sheetId="1" r:id="rId1"/>
+  </sheets>
+</workbook>
 </file>
</xml_diff>